<commit_message>
labels and notebook logic
</commit_message>
<xml_diff>
--- a/data/processed/day4_label_sheet_pass1.xlsx
+++ b/data/processed/day4_label_sheet_pass1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="labels" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="labels" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Air Traffic Controllers Start Resigning as Shutdown Bites. | Unpaid air traffic controllers are quitting their jobs altogether as the longest government shutdown in U.S. history continues.</t>
+          <t>Hey No Kings: If corporate media heavily hypes your protest movement, it's not a protest movement</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr"/>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Democratic Centrists Want to Fight—and Prove They Will Take on the Establishment | Crop of moderate Democrats trying to counter Trump and progressive influence in their own party</t>
+          <t>Opposition to single-payer healthcare separates Villaraigosa from others at candidate forum</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr"/>
@@ -3067,7 +3067,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Harmeet Dhillon Was an Outspoken Advocate for the Right of States to Run Elections. Then She Took a Top Job at Trump’s DOJ</t>
+          <t>Moderate Democrats say they'd save Speaker Mike Johnson if the right tries to oust him</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr"/>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Kamala Harris says she will cut degree requirements for certain federal jobs</t>
+          <t>Trump's gold shoes ridiculed after price drop: 'Just surrendered 75% of their price'</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr"/>
@@ -4327,7 +4327,7 @@
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>The impossible math behind Trump's $2,000 tariff rebate plan | About That</t>
+          <t>Dems Struggle to Make Their Moderates Go Viral: Searching for a candidate who can be Mamdani in the streets and Manchin in the seats.</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr"/>
@@ -4456,7 +4456,7 @@
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Trump downplays recession fears, saying the U.S. would be 'OK' in the long term</t>
+          <t>Federal employees ordered to remove pronouns from their email signature and urged to find ‘higher productivity jobs’</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr"/>
@@ -4682,7 +4682,7 @@
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>Trump's gold shoes ridiculed after price drop: 'Just surrendered 75% of their price'</t>
+          <t>UAW clinches watershed union victory at Volkswagen Tennessee factory</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr"/>
@@ -7123,7 +7123,7 @@
       </c>
       <c r="B268" s="2" t="inlineStr">
         <is>
-          <t>In case you didn't know, the President doesn't control gas prices.</t>
+          <t>Marjorie Taylor Greene Calls Out Trump’s Blatant Lie on Inflation</t>
         </is>
       </c>
       <c r="C268" s="2" t="inlineStr"/>

</xml_diff>